<commit_message>
test data and pages
</commit_message>
<xml_diff>
--- a/test data/SauceDemoTestData.xlsx
+++ b/test data/SauceDemoTestData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" state="visible" r:id="rId1"/>
@@ -209,13 +209,10 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -720,7 +717,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col bestFit="1" customWidth="1" min="1" max="1" width="13.5546875"/>
-    <col bestFit="1" customWidth="1" min="2" max="2" width="14.6640625"/>
+    <col customWidth="1" min="2" max="2" width="17.8515625"/>
     <col bestFit="1" customWidth="1" min="3" max="3" width="11.6640625"/>
     <col bestFit="1" customWidth="1" min="4" max="4" width="13.88671875"/>
     <col bestFit="1" customWidth="1" min="5" max="5" width="17.88671875"/>
@@ -1028,10 +1025,10 @@
       <c r="D2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>42</v>
       </c>
       <c r="G2" s="2">
@@ -1057,10 +1054,10 @@
       <c r="D3" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>41</v>
       </c>
       <c r="G3" s="2">

</xml_diff>